<commit_message>
crea documentos y modifica barras
</commit_message>
<xml_diff>
--- a/documentos/CARGUE INICIAL RFID.xlsx
+++ b/documentos/CARGUE INICIAL RFID.xlsx
@@ -4,19 +4,17 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19815" windowHeight="7815" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12495" tabRatio="585"/>
   </bookViews>
   <sheets>
     <sheet name="cargue masivo" sheetId="1" r:id="rId1"/>
-    <sheet name="cargue items" sheetId="2" r:id="rId2"/>
-    <sheet name="cargue ubicaciones y zonas" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>item</t>
   </si>
@@ -78,16 +76,22 @@
     <t>ENDURO</t>
   </si>
   <si>
-    <t>Sede 1</t>
+    <t>001</t>
+  </si>
+  <si>
+    <t>Principal</t>
   </si>
   <si>
     <t>Cali</t>
   </si>
   <si>
-    <t>flora</t>
-  </si>
-  <si>
-    <t>Bodega principal</t>
+    <t>calle 38a 4n 183</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>piso 1</t>
   </si>
   <si>
     <t>LLANTA KENDA KD1002</t>
@@ -102,13 +106,10 @@
     <t>PISTA</t>
   </si>
   <si>
-    <t>codigo Ubicacion</t>
-  </si>
-  <si>
-    <t>codigo zona</t>
-  </si>
-  <si>
-    <t>descripcion zona</t>
+    <t>03</t>
+  </si>
+  <si>
+    <t>pdv</t>
   </si>
 </sst>
 </file>
@@ -116,9 +117,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="20">
@@ -130,6 +131,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="3"/>
@@ -145,8 +160,25 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -154,36 +186,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -230,6 +232,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -246,14 +255,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -261,20 +262,20 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -283,61 +284,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -349,127 +476,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -480,6 +487,41 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -502,22 +544,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -525,8 +552,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -546,17 +573,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -571,27 +587,18 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -606,22 +613,22 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -630,111 +637,114 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="19" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
@@ -1076,22 +1086,22 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
@@ -1100,10 +1110,10 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -1123,7 +1133,7 @@
       <c r="B2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D2" t="s">
@@ -1141,23 +1151,23 @@
       <c r="H2">
         <v>17</v>
       </c>
-      <c r="J2">
-        <v>1</v>
+      <c r="J2" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="K2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2">
-        <v>1010</v>
+        <v>23</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>24</v>
       </c>
       <c r="O2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="P2">
         <v>100</v>
@@ -1168,16 +1178,16 @@
         <v>1002</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F3">
         <v>90</v>
@@ -1188,105 +1198,26 @@
       <c r="H3">
         <v>17</v>
       </c>
-      <c r="J3">
-        <v>1</v>
+      <c r="J3" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3">
-        <v>1010</v>
+        <v>23</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="O3" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="P3">
         <v>50</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="1"/>
-  <cols>
-    <col min="2" max="2" width="24.1428571428571" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2">
-        <v>1005</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3">
-        <v>1002</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
-  <cols>
-    <col min="1" max="1" width="17.2857142857143" customWidth="1"/>
-    <col min="2" max="2" width="11.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="7.42857142857143" customWidth="1"/>
-    <col min="4" max="4" width="9.71428571428571" customWidth="1"/>
-    <col min="5" max="5" width="12.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>